<commit_message>
Pushing updated files from streams.
</commit_message>
<xml_diff>
--- a/_Projects/P1012202501-ESP32_Stepper_Controller/ProjectDocuments/P1012202501-Project_Budget.xlsx
+++ b/_Projects/P1012202501-ESP32_Stepper_Controller/ProjectDocuments/P1012202501-Project_Budget.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="30">
   <si>
     <t xml:space="preserve">Materials Budget:</t>
   </si>
@@ -107,6 +107,9 @@
   </si>
   <si>
     <t xml:space="preserve">Digikey Taxes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variable Power Resistor</t>
   </si>
 </sst>
 </file>
@@ -489,7 +492,7 @@
       <c r="B2" s="1"/>
       <c r="C2" s="2" t="n">
         <f aca="false">SUM(E10:E53)</f>
-        <v>684.95</v>
+        <v>719.95</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>3</v>
@@ -508,7 +511,7 @@
       <c r="B3" s="1"/>
       <c r="C3" s="2" t="n">
         <f aca="false">C1-C2</f>
-        <v>1315.05</v>
+        <v>1280.05</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>5</v>
@@ -1283,13 +1286,19 @@
       <c r="M45" s="8"/>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="5"/>
+      <c r="A46" s="5" t="s">
+        <v>29</v>
+      </c>
       <c r="B46" s="5"/>
-      <c r="C46" s="6"/>
-      <c r="D46" s="2"/>
+      <c r="C46" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>35</v>
+      </c>
       <c r="E46" s="2" t="n">
         <f aca="false">C46*D46</f>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F46" s="3"/>
       <c r="G46" s="8"/>

</xml_diff>

<commit_message>
Added new items from recent stream.
</commit_message>
<xml_diff>
--- a/_Projects/P1012202501-ESP32_Stepper_Controller/ProjectDocuments/P1012202501-Project_Budget.xlsx
+++ b/_Projects/P1012202501-ESP32_Stepper_Controller/ProjectDocuments/P1012202501-Project_Budget.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="39">
   <si>
     <t xml:space="preserve">Materials Budget:</t>
   </si>
@@ -91,9 +91,6 @@
     <t xml:space="preserve">Mouser Duty Fee</t>
   </si>
   <si>
-    <t xml:space="preserve">Mouser Taxes</t>
-  </si>
-  <si>
     <t xml:space="preserve">DigiKey Components</t>
   </si>
   <si>
@@ -110,6 +107,36 @@
   </si>
   <si>
     <t xml:space="preserve">Variable Power Resistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panel Ammeter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enclosure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Switch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Power Adapter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Power Connector</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Banana Plugs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Connectors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nylon Standoffs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mouser – Light Pipes</t>
   </si>
 </sst>
 </file>
@@ -465,7 +492,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M48"/>
+  <dimension ref="A1:M61"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -491,8 +518,8 @@
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="2" t="n">
-        <f aca="false">SUM(E10:E53)</f>
-        <v>719.95</v>
+        <f aca="false">SUM(E10:E89)</f>
+        <v>906.14</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>3</v>
@@ -500,7 +527,7 @@
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
       <c r="H2" s="3" t="n">
-        <f aca="false">SUM(F10:F58)</f>
+        <f aca="false">SUM(F10:F57)</f>
         <v>0</v>
       </c>
     </row>
@@ -511,7 +538,7 @@
       <c r="B3" s="1"/>
       <c r="C3" s="2" t="n">
         <f aca="false">C1-C2</f>
-        <v>1280.05</v>
+        <v>1093.86</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>5</v>
@@ -1127,10 +1154,12 @@
       <c r="C39" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D39" s="2"/>
+      <c r="D39" s="2" t="n">
+        <v>8.12</v>
+      </c>
       <c r="E39" s="2" t="n">
         <f aca="false">C39*D39</f>
-        <v>0</v>
+        <v>8.12</v>
       </c>
       <c r="F39" s="3"/>
       <c r="G39" s="8"/>
@@ -1150,11 +1179,11 @@
         <v>1</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>8.12</v>
+        <v>6.99</v>
       </c>
       <c r="E40" s="2" t="n">
         <f aca="false">C40*D40</f>
-        <v>8.12</v>
+        <v>6.99</v>
       </c>
       <c r="F40" s="3"/>
       <c r="G40" s="8"/>
@@ -1174,11 +1203,11 @@
         <v>1</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>6.99</v>
+        <v>1.02</v>
       </c>
       <c r="E41" s="2" t="n">
         <f aca="false">C41*D41</f>
-        <v>6.99</v>
+        <v>1.02</v>
       </c>
       <c r="F41" s="3"/>
       <c r="G41" s="8"/>
@@ -1198,11 +1227,11 @@
         <v>1</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>1.02</v>
+        <v>15.64</v>
       </c>
       <c r="E42" s="2" t="n">
         <f aca="false">C42*D42</f>
-        <v>1.02</v>
+        <v>15.64</v>
       </c>
       <c r="F42" s="3"/>
       <c r="G42" s="8"/>
@@ -1222,11 +1251,11 @@
         <v>1</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>15.64</v>
+        <v>1.06</v>
       </c>
       <c r="E43" s="2" t="n">
         <f aca="false">C43*D43</f>
-        <v>15.64</v>
+        <v>1.06</v>
       </c>
       <c r="F43" s="3"/>
       <c r="G43" s="8"/>
@@ -1237,20 +1266,20 @@
       <c r="L43" s="8"/>
       <c r="M43" s="8"/>
     </row>
-    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B44" s="5"/>
       <c r="C44" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>1.06</v>
+        <v>6.99</v>
       </c>
       <c r="E44" s="2" t="n">
         <f aca="false">C44*D44</f>
-        <v>1.06</v>
+        <v>6.99</v>
       </c>
       <c r="F44" s="3"/>
       <c r="G44" s="8"/>
@@ -1263,18 +1292,18 @@
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B45" s="5"/>
       <c r="C45" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>6.99</v>
+        <v>35</v>
       </c>
       <c r="E45" s="2" t="n">
         <f aca="false">C45*D45</f>
-        <v>6.99</v>
+        <v>35</v>
       </c>
       <c r="F45" s="3"/>
       <c r="G45" s="8"/>
@@ -1294,11 +1323,11 @@
         <v>1</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="E46" s="2" t="n">
         <f aca="false">C46*D46</f>
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="F46" s="3"/>
       <c r="G46" s="8"/>
@@ -1310,13 +1339,19 @@
       <c r="M46" s="8"/>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="5"/>
+      <c r="A47" s="5" t="s">
+        <v>30</v>
+      </c>
       <c r="B47" s="5"/>
-      <c r="C47" s="6"/>
-      <c r="D47" s="2"/>
+      <c r="C47" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>23.99</v>
+      </c>
       <c r="E47" s="2" t="n">
         <f aca="false">C47*D47</f>
-        <v>0</v>
+        <v>23.99</v>
       </c>
       <c r="F47" s="3"/>
       <c r="G47" s="8"/>
@@ -1328,13 +1363,19 @@
       <c r="M47" s="8"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="5"/>
+      <c r="A48" s="5" t="s">
+        <v>31</v>
+      </c>
       <c r="B48" s="5"/>
-      <c r="C48" s="6"/>
-      <c r="D48" s="2"/>
+      <c r="C48" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>17.95</v>
+      </c>
       <c r="E48" s="2" t="n">
         <f aca="false">C48*D48</f>
-        <v>0</v>
+        <v>17.95</v>
       </c>
       <c r="F48" s="3"/>
       <c r="G48" s="8"/>
@@ -1345,8 +1386,290 @@
       <c r="L48" s="8"/>
       <c r="M48" s="8"/>
     </row>
+    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B49" s="5"/>
+      <c r="C49" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="2" t="n">
+        <v>6.39</v>
+      </c>
+      <c r="E49" s="2" t="n">
+        <f aca="false">C49*D49</f>
+        <v>6.39</v>
+      </c>
+      <c r="F49" s="3"/>
+      <c r="G49" s="8"/>
+      <c r="H49" s="8"/>
+      <c r="I49" s="8"/>
+      <c r="J49" s="8"/>
+      <c r="K49" s="8"/>
+      <c r="L49" s="8"/>
+      <c r="M49" s="8"/>
+    </row>
+    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B50" s="5"/>
+      <c r="C50" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>7.97</v>
+      </c>
+      <c r="E50" s="2" t="n">
+        <f aca="false">C50*D50</f>
+        <v>7.97</v>
+      </c>
+      <c r="F50" s="3"/>
+      <c r="G50" s="8"/>
+      <c r="H50" s="8"/>
+      <c r="I50" s="8"/>
+      <c r="J50" s="8"/>
+      <c r="K50" s="8"/>
+      <c r="L50" s="8"/>
+      <c r="M50" s="8"/>
+    </row>
+    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B51" s="5"/>
+      <c r="C51" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" s="2" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="E51" s="2" t="n">
+        <f aca="false">C51*D51</f>
+        <v>5.99</v>
+      </c>
+      <c r="F51" s="3"/>
+      <c r="G51" s="8"/>
+      <c r="H51" s="8"/>
+      <c r="I51" s="8"/>
+      <c r="J51" s="8"/>
+      <c r="K51" s="8"/>
+      <c r="L51" s="8"/>
+      <c r="M51" s="8"/>
+    </row>
+    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B52" s="5"/>
+      <c r="C52" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>10.49</v>
+      </c>
+      <c r="E52" s="2" t="n">
+        <f aca="false">C52*D52</f>
+        <v>20.98</v>
+      </c>
+      <c r="F52" s="3"/>
+      <c r="G52" s="8"/>
+      <c r="H52" s="8"/>
+      <c r="I52" s="8"/>
+      <c r="J52" s="8"/>
+      <c r="K52" s="8"/>
+      <c r="L52" s="8"/>
+      <c r="M52" s="8"/>
+    </row>
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B53" s="5"/>
+      <c r="C53" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>16.99</v>
+      </c>
+      <c r="E53" s="2" t="n">
+        <f aca="false">C53*D53</f>
+        <v>50.97</v>
+      </c>
+      <c r="F53" s="3"/>
+      <c r="G53" s="8"/>
+      <c r="H53" s="8"/>
+      <c r="I53" s="8"/>
+      <c r="J53" s="8"/>
+      <c r="K53" s="8"/>
+      <c r="L53" s="8"/>
+      <c r="M53" s="8"/>
+    </row>
+    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B54" s="5"/>
+      <c r="C54" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="E54" s="2" t="n">
+        <f aca="false">C54*D54</f>
+        <v>20</v>
+      </c>
+      <c r="F54" s="3"/>
+      <c r="G54" s="8"/>
+      <c r="H54" s="8"/>
+      <c r="I54" s="8"/>
+      <c r="J54" s="8"/>
+      <c r="K54" s="8"/>
+      <c r="L54" s="8"/>
+      <c r="M54" s="8"/>
+    </row>
+    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B55" s="5"/>
+      <c r="C55" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" s="2" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="E55" s="2" t="n">
+        <f aca="false">C55*D55</f>
+        <v>6.99</v>
+      </c>
+      <c r="F55" s="3"/>
+      <c r="G55" s="8"/>
+      <c r="H55" s="8"/>
+      <c r="I55" s="8"/>
+      <c r="J55" s="8"/>
+      <c r="K55" s="8"/>
+      <c r="L55" s="8"/>
+      <c r="M55" s="8"/>
+    </row>
+    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B56" s="5"/>
+      <c r="C56" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>15.96</v>
+      </c>
+      <c r="E56" s="2" t="n">
+        <f aca="false">C56*D56</f>
+        <v>15.96</v>
+      </c>
+      <c r="F56" s="3"/>
+      <c r="G56" s="8"/>
+      <c r="H56" s="8"/>
+      <c r="I56" s="8"/>
+      <c r="J56" s="8"/>
+      <c r="K56" s="8"/>
+      <c r="L56" s="8"/>
+      <c r="M56" s="8"/>
+    </row>
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="5"/>
+      <c r="B57" s="5"/>
+      <c r="C57" s="6"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2" t="n">
+        <f aca="false">C57*D57</f>
+        <v>0</v>
+      </c>
+      <c r="F57" s="3"/>
+      <c r="G57" s="8"/>
+      <c r="H57" s="8"/>
+      <c r="I57" s="8"/>
+      <c r="J57" s="8"/>
+      <c r="K57" s="8"/>
+      <c r="L57" s="8"/>
+      <c r="M57" s="8"/>
+    </row>
+    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="5"/>
+      <c r="B58" s="5"/>
+      <c r="C58" s="6"/>
+      <c r="D58" s="2"/>
+      <c r="E58" s="2" t="n">
+        <f aca="false">C58*D58</f>
+        <v>0</v>
+      </c>
+      <c r="F58" s="3"/>
+      <c r="G58" s="8"/>
+      <c r="H58" s="8"/>
+      <c r="I58" s="8"/>
+      <c r="J58" s="8"/>
+      <c r="K58" s="8"/>
+      <c r="L58" s="8"/>
+      <c r="M58" s="8"/>
+    </row>
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="5"/>
+      <c r="B59" s="5"/>
+      <c r="C59" s="6"/>
+      <c r="D59" s="2"/>
+      <c r="E59" s="2" t="n">
+        <f aca="false">C59*D59</f>
+        <v>0</v>
+      </c>
+      <c r="F59" s="3"/>
+      <c r="G59" s="8"/>
+      <c r="H59" s="8"/>
+      <c r="I59" s="8"/>
+      <c r="J59" s="8"/>
+      <c r="K59" s="8"/>
+      <c r="L59" s="8"/>
+      <c r="M59" s="8"/>
+    </row>
+    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="5"/>
+      <c r="B60" s="5"/>
+      <c r="C60" s="6"/>
+      <c r="D60" s="2"/>
+      <c r="E60" s="2" t="n">
+        <f aca="false">C60*D60</f>
+        <v>0</v>
+      </c>
+      <c r="F60" s="3"/>
+      <c r="G60" s="8"/>
+      <c r="H60" s="8"/>
+      <c r="I60" s="8"/>
+      <c r="J60" s="8"/>
+      <c r="K60" s="8"/>
+      <c r="L60" s="8"/>
+      <c r="M60" s="8"/>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="5"/>
+      <c r="B61" s="5"/>
+      <c r="C61" s="6"/>
+      <c r="D61" s="2"/>
+      <c r="E61" s="2" t="n">
+        <f aca="false">C61*D61</f>
+        <v>0</v>
+      </c>
+      <c r="F61" s="3"/>
+      <c r="G61" s="8"/>
+      <c r="H61" s="8"/>
+      <c r="I61" s="8"/>
+      <c r="J61" s="8"/>
+      <c r="K61" s="8"/>
+      <c r="L61" s="8"/>
+      <c r="M61" s="8"/>
+    </row>
   </sheetData>
-  <mergeCells count="87">
+  <mergeCells count="113">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="E1:G1"/>
     <mergeCell ref="A2:B2"/>
@@ -1434,6 +1757,32 @@
     <mergeCell ref="G47:M47"/>
     <mergeCell ref="A48:B48"/>
     <mergeCell ref="G48:M48"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="G49:M49"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="G50:M50"/>
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="G51:M51"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="G52:M52"/>
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="G53:M53"/>
+    <mergeCell ref="A54:B54"/>
+    <mergeCell ref="G54:M54"/>
+    <mergeCell ref="A55:B55"/>
+    <mergeCell ref="G55:M55"/>
+    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="G56:M56"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="G57:M57"/>
+    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="G58:M58"/>
+    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="G59:M59"/>
+    <mergeCell ref="A60:B60"/>
+    <mergeCell ref="G60:M60"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="G61:M61"/>
   </mergeCells>
   <conditionalFormatting sqref="C3">
     <cfRule type="cellIs" priority="2" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">

</xml_diff>